<commit_message>
Updated it to read excel sheet using Uipath and automatically update the inventory.
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -19,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,21 +29,33 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -53,21 +64,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
+        <fgColor rgb="FF1E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF2FF"/>
+        <fgColor rgb="FFEEF2FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="FF1E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF22C55E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -77,23 +103,35 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -116,16 +154,36 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -488,8 +546,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -524,6 +582,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -547,83 +610,182 @@
           <t>electronic modern</t>
         </is>
       </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Wireless Handfree</t>
+          <t>Keyboard</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>electronic</t>
         </is>
       </c>
       <c r="C3" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="E3" s="5" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>normal one</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Wireless Mouse</t>
+          <t>Marker Pen</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+        <v>0.25</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Sri Lankan Product</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>mobile phone</t>
+          <t>Smart Board</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>electronic</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>155</v>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>chinese</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr"/>
-      <c r="C6" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>230.25</v>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Wireless Mouse</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Headset XXV</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>ccvv</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Last updated: 2026-06-08 14:58:04</t>
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Laptop HP</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Electronic</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>114</v>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Sl111</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Last updated: 2026-06-09 10:31:39</t>
         </is>
       </c>
     </row>

</xml_diff>